<commit_message>
xlsx: rename 3.1.2a to clarify apprentice cohort
Project 3.1 and 3.1.2a both had the title "CPL Offers & Awards
Tracking" — confusing in the dashboard's projects grid (two cards with
identical names). They're NOT duplicates: each tracks a distinct KPI
series:

  - 3.1   → cumulative Californians served with CPL (target: 250k by 2030)
  - 3.1.2a → cumulative apprentices + journey workers served with CPL
            (target: 20k by 2030)

Renaming 3.1.2a → "CPL Offers & Awards Tracking — Apprentice Cohort"
preserves both KPI progress bars and removes the duplicate-card
confusion. No structural change; all other fields (activity, goal,
lead, budget, dates, targets) unchanged.

CPL_Data.js will be regenerated by the daily cron — not committed here
to keep the diff scope clean.
</commit_message>
<xml_diff>
--- a/CPL_Initiative_Project_List_v3.xlsx
+++ b/CPL_Initiative_Project_List_v3.xlsx
@@ -2464,7 +2464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG52"/>
+  <dimension ref="A1:AD52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="16" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="6" customWidth="1" style="187" min="1" max="1"/>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="B15" s="171" t="inlineStr">
         <is>
-          <t>CPL Offers &amp; Awards Tracking</t>
+          <t>CPL Offers &amp; Awards Tracking — Apprentice Cohort</t>
         </is>
       </c>
       <c r="C15" s="172" t="inlineStr">

</xml_diff>

<commit_message>
xlsx: rename 3.1 cohort family to disambiguate cards
Activity 3 had four project cards titled "CPL Offers & Awards
Tracking" — 3.1 (all populations), 3.1.1 (working adults), 3.1.2
(veterans), 3.1.2a (apprentices). PR #142 disambiguated 3.1.2a only;
this finishes the family.

Renames:
  3.1    -> CPL Offers & Awards Tracking — All Populations
  3.1.1  -> CPL Offers & Awards Tracking — Working Adults
  3.1.2  -> CPL Offers & Awards Tracking — Veterans & Service Members
  3.1.2a -> (unchanged) Apprentice Cohort

All four track distinct KPI series (per-cohort goal/stretch ladders),
so disambiguation is the right move — folding would have lost the
per-cohort progress bars.

CPL_Data.js intentionally not committed; daily cron will regenerate.
</commit_message>
<xml_diff>
--- a/CPL_Initiative_Project_List_v3.xlsx
+++ b/CPL_Initiative_Project_List_v3.xlsx
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B12" s="171" t="inlineStr">
         <is>
-          <t>CPL Offers &amp; Awards Tracking</t>
+          <t>CPL Offers &amp; Awards Tracking — All Populations</t>
         </is>
       </c>
       <c r="C12" s="172" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="B13" s="171" t="inlineStr">
         <is>
-          <t>CPL Offers &amp; Awards Tracking</t>
+          <t>CPL Offers &amp; Awards Tracking — Working Adults</t>
         </is>
       </c>
       <c r="C13" s="172" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="B14" s="171" t="inlineStr">
         <is>
-          <t>CPL Offers &amp; Awards Tracking</t>
+          <t>CPL Offers &amp; Awards Tracking — Veterans &amp; Service Members</t>
         </is>
       </c>
       <c r="C14" s="172" t="inlineStr">

</xml_diff>